<commit_message>
docs: update documentation for agentification support
</commit_message>
<xml_diff>
--- a/assets/core/files/_metadata.xlsx
+++ b/assets/core/files/_metadata.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charnould/GitHub/pierre/assets/default/files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charnould/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6723546E-73EA-1140-BD6C-E9E2CBE46E2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{287A388B-179D-3A43-9281-1B9D7F5B3C87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{E5B0FB10-8797-D243-A0FA-6D923D5CC0EA}"/>
+    <workbookView xWindow="860" yWindow="1320" windowWidth="26420" windowHeight="14440" xr2:uid="{E5B0FB10-8797-D243-A0FA-6D923D5CC0EA}"/>
   </bookViews>
   <sheets>
     <sheet name="metadata" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">metadata!$A$3:$G$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">metadata!$A$3:$E$3</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,16 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
-  <si>
-    <t>true</t>
-  </si>
-  <si>
-    <t>Ci-après la description et les caractéristiques techniques d'une résidence de Pierre Habitat :</t>
-  </si>
-  <si>
-    <t>Ci-après les noms et coordonnées des collaborateurs en charge des résidences chez Pierre Habitat :</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
   <si>
     <t>filename</t>
   </si>
@@ -62,22 +53,12 @@
     <t>headers</t>
   </si>
   <si>
-    <t>chunk</t>
-  </si>
-  <si>
-    <t>group_by</t>
+    <t>agent_filename</t>
   </si>
   <si>
     <t xml:space="preserve">
-Indiquer à quelle ligne se trouve la ligne d'en-têtes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Indiquer l'onglet concerné.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Parfois, il est pertinent de considérer un fichier Excel non pas ligne à ligne, mais comme un bloc. Mettre « false » pour que le tableau soit stocké en un bloc.</t>
+Indiquer l'onglet concerné.
+</t>
   </si>
   <si>
     <r>
@@ -88,7 +69,7 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <rFont val="Arial"/>
+        <rFont val="Helvetica"/>
         <family val="2"/>
       </rPr>
       <t>exactement</t>
@@ -96,87 +77,13 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <rFont val="Arial"/>
+        <rFont val="Helvetica"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> au nom du fichier uploadé. Respecter les espaces et la casse.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-Optionnel.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Quelle colonne peut-on utiliser pour grouper les résultats ?</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">
-Optionnel mais </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>important</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">. 
-Afin d'aider PIERRE à comprendre le sujet couvert par l'onglet, indiquer avec les mots-clefs les plus pertinents à quoi correspond </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>une ligne du fichier Excel.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Applicable uniquement aux fichiers .XLSX (Excel). </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="9" tint="-0.249977111117893"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Sans effet pour les fichiers .DOCX (Word) et .MD (Markdown).</t>
-    </r>
-  </si>
-  <si>
-    <t>exemple.xlsx</t>
-  </si>
-  <si>
-    <t>exemple.docx</t>
-  </si>
-  <si>
-    <t>description</t>
+      <t xml:space="preserve"> au nom du fichier uploadé.
+Respecter les espaces et la casse.
+</t>
+    </r>
   </si>
   <si>
     <r>
@@ -215,18 +122,118 @@
         <rFont val="Helvetica"/>
         <family val="2"/>
       </rPr>
-      <t>.
-Les profils sont ceux définis dans le fichier relatif aux utilisateurs.</t>
-    </r>
-  </si>
-  <si>
-    <t>agent_astreinte, cadre_astreinte</t>
-  </si>
-  <si>
-    <t>cadre_astreinte, agent_jour</t>
-  </si>
-  <si>
-    <t>agent_jour</t>
+      <t xml:space="preserve">.
+Les profils sont ceux définis dans le fichier relatif aux utilisateurs.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">
+Obligatoire et </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>TRÈS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>important</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">.
+Afin d'aider PIERRE à comprendre le sujet couvert par le fichier/onglet, nommer ici le document avec un titre explicite En effet, PIERRE réfléchit à quels documents consulter sur la base des noms indiqués ci-dessous.
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Applicable uniquement aux fichiers Excel. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF3C7D22"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t>Sans effet sur les autres types de fichiers.</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF3C7D22"/>
+        <rFont val="Helvetica"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Indiquer à quelle ligne se trouve les en-têtes.
+</t>
+  </si>
+  <si>
+    <t>Histoire de l'OPH du Vaucluse</t>
+  </si>
+  <si>
+    <t>agent, cadre</t>
+  </si>
+  <si>
+    <t>default, agent, cadre</t>
+  </si>
+  <si>
+    <t>Bonnes pratiques pour les agents d'accueil</t>
+  </si>
+  <si>
+    <t>Bonnes pratiques pour les agents d'accueil.docx</t>
+  </si>
+  <si>
+    <t>Histoire de l'OPH du Vaucluse.docx</t>
+  </si>
+  <si>
+    <t>agent</t>
+  </si>
+  <si>
+    <t>Cahier de consignes.xlsx</t>
+  </si>
+  <si>
+    <t>Procédures et responsabilités des agents de jour</t>
+  </si>
+  <si>
+    <t>Procédures et responsabilités des agents d'astreinte</t>
+  </si>
+  <si>
+    <t>pat_extract.xlsx</t>
+  </si>
+  <si>
+    <t>Description et caractéristiques techniques du patrimoine</t>
   </si>
 </sst>
 </file>
@@ -247,32 +254,7 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
       <sz val="12"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="9" tint="-0.249977111117893"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="9" tint="-0.249977111117893"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -288,13 +270,38 @@
       <family val="2"/>
     </font>
     <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Helvetica"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3C7D22"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3C7D22"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -303,38 +310,50 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FFDAE9F8"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FFCAEDFB"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FFDAF2D0"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FFA6C9EC"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.749992370372631"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FF94DCF8"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.89999084444715716"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FFB5E6A2"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
@@ -350,40 +369,52 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -719,147 +750,352 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F3359B2-613C-1246-BB58-A3F329ACACAC}">
-  <dimension ref="A1:G6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24.5" style="1" customWidth="1"/>
-    <col min="2" max="2" width="34.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.33203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="21.6640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="25.1640625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="28.83203125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="102.6640625" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="1" width="63.5" style="2" customWidth="1"/>
+    <col min="2" max="2" width="60.33203125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="24.6640625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="71.5" style="2" customWidth="1"/>
+    <col min="6" max="16384" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:6" ht="68" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="14"/>
+      <c r="E1" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:6" s="5" customFormat="1" ht="73" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="12"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" s="15"/>
+      <c r="F2" s="4"/>
+    </row>
+    <row r="3" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="1"/>
+    </row>
+    <row r="4" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="1"/>
+    </row>
+    <row r="5" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="1"/>
+    </row>
+    <row r="6" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="C6" s="11">
+        <v>1</v>
+      </c>
+      <c r="D6" s="11">
+        <v>1</v>
+      </c>
+      <c r="E6" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
+      <c r="F6" s="1"/>
     </row>
-    <row r="2" spans="1:7" s="2" customFormat="1" ht="106" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="8"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>14</v>
-      </c>
+    <row r="7" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="11">
+        <v>2</v>
+      </c>
+      <c r="D7" s="11">
+        <v>1</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="1"/>
     </row>
-    <row r="3" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+    <row r="8" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="11">
         <v>3</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="1">
-        <v>1</v>
-      </c>
-      <c r="D4" s="1">
-        <v>3</v>
-      </c>
-      <c r="E4" s="1">
-        <v>1</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="1">
+      <c r="D8" s="11">
         <v>2</v>
       </c>
-      <c r="D5" s="1">
-        <v>1</v>
-      </c>
-      <c r="E5" s="1">
-        <v>6</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" s="1" t="s">
+      <c r="E8" s="10" t="s">
         <v>22</v>
       </c>
+      <c r="F8" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:G3" xr:uid="{0F3359B2-613C-1246-BB58-A3F329ACACAC}"/>
+  <autoFilter ref="A3:E8" xr:uid="{0F3359B2-613C-1246-BB58-A3F329ACACAC}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:E8">
+      <sortCondition ref="A3:A8"/>
+    </sortState>
+  </autoFilter>
   <dataConsolidate/>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:G1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="E1:E2"/>
   </mergeCells>
-  <dataValidations count="2">
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F997:F1675 D4:D1675" xr:uid="{49006576-7484-B84D-A51B-69FE1DA1041A}">
+  <dataValidations count="1">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D9:D1595" xr:uid="{49006576-7484-B84D-A51B-69FE1DA1041A}">
       <formula1>1</formula1>
       <formula2>10</formula2>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F4:F996" xr:uid="{1B35C915-B844-3A4E-8381-4D4F9C183493}">
-      <formula1>"true,false"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010007C0A6F2F814D741ADAAB1D4BE61BFBF" ma:contentTypeVersion="3" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="6080c67114cd18bfa711ced86a8ee399">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="95589ea0-eb1b-4a66-97f4-667092e2579b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ef73da726e8c35c4a1674bf6af49a8cc" ns2:_="">
+    <xsd:import namespace="95589ea0-eb1b-4a66-97f4-667092e2579b"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="95589ea0-eb1b-4a66-97f4-667092e2579b" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Type de contenu"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titre"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F78FBE11-2A0A-4C6F-8B1F-8A4D454F9E5B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="95589ea0-eb1b-4a66-97f4-667092e2579b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C8704A3-4697-4081-95E7-11F6FAC0ADC3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9E04CA4-A95F-40C5-A339-7D19A06C86AB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>